<commit_message>
Subindo casos de testes.
</commit_message>
<xml_diff>
--- a/documentação/Testes/Caso de Teste/UC13  - EXIBIR PRONTUÁRIO.xlsx
+++ b/documentação/Testes/Caso de Teste/UC13  - EXIBIR PRONTUÁRIO.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Casos de Teste" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Casos de Teste" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="58">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -355,13 +355,119 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="32.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="32.2421875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.04"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="2" style="2" width="32.22"/>
@@ -429,6 +535,9 @@
       <c r="E3" s="6" t="s">
         <v>17</v>
       </c>
+      <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -446,6 +555,9 @@
       <c r="E4" s="6" t="s">
         <v>22</v>
       </c>
+      <c r="F4" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -463,6 +575,9 @@
       <c r="E5" s="6" t="s">
         <v>27</v>
       </c>
+      <c r="F5" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -480,6 +595,9 @@
       <c r="E6" s="6" t="s">
         <v>32</v>
       </c>
+      <c r="F6" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
@@ -497,6 +615,9 @@
       <c r="E7" s="6" t="s">
         <v>37</v>
       </c>
+      <c r="F7" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
@@ -514,6 +635,9 @@
       <c r="E8" s="6" t="s">
         <v>42</v>
       </c>
+      <c r="F8" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
@@ -531,6 +655,9 @@
       <c r="E9" s="6" t="s">
         <v>47</v>
       </c>
+      <c r="F9" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -548,6 +675,9 @@
       </c>
       <c r="E10" s="6" t="s">
         <v>52</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>